<commit_message>
feat(snr): accrual basis from 2026-07 — revenue earned in M, paid in M+1; July frozen at 10,517,426 (#174)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-07/skybase_settlement_july_2026.xlsx
+++ b/settlements/skybase/2026-07/skybase_settlement_july_2026.xlsx
@@ -513,17 +513,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>+ governance_accessibility_rewards (0.01 × SNR 2026-07 = 15225588.80793415141613319624 (sky_total generated sky_total))</t>
+          <t>+ governance_accessibility_rewards (0.01 × SNR 2026-07 = 10517425.807934152 (sky_total generated 2026-08-07T11:52:07+00:00))</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>152255.8880793415</v>
+        <v>105174.2580793415</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" s="4" t="n">
-        <v>285188.5181444788</v>
+        <v>238106.8881444788</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-06T00:02:57+00:00</t>
+          <t>2026-08-07T11:52:24+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>